<commit_message>
Complete Railway→Fly migration: all docs, numbers, Memo sync
</commit_message>
<xml_diff>
--- a/files/confidential/Numbers.xlsx
+++ b/files/confidential/Numbers.xlsx
@@ -878,15 +878,15 @@
     <row r="32">
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Railway</t>
+          <t>Fly.io</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>railway.com</t>
+          <t>fly.io</t>
         </is>
       </c>
     </row>

</xml_diff>